<commit_message>
Actividad 1 primer borrador
</commit_message>
<xml_diff>
--- a/data/outputs/sectores_priorizados.xlsx
+++ b/data/outputs/sectores_priorizados.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="88">
   <si>
     <t xml:space="preserve">criterio</t>
   </si>
@@ -143,25 +143,43 @@
     <t xml:space="preserve">Inversión</t>
   </si>
   <si>
+    <t xml:space="preserve">FBKF estimada, máximo de los dos métodos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Baja</t>
+  </si>
+  <si>
+    <t xml:space="preserve">c07 y c09</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FBKF estimada, mínimo de los dos métodos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FBKF estimada, valor central</t>
+  </si>
+  <si>
     <t xml:space="preserve">IED, flujo acumulado 2022-2024</t>
   </si>
   <si>
-    <t xml:space="preserve">Baja</t>
+    <t xml:space="preserve">IED, posición al cierre</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tasa de inversión (FBKF sobre valor agregado)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">% (media 2022-2024)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Concentración de mercado</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Empresas en la sección CIIU principal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">empresas (2022)</t>
   </si>
   <si>
     <t xml:space="preserve">c07</t>
-  </si>
-  <si>
-    <t xml:space="preserve">IED, posición al cierre</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Concentración de mercado</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Empresas en la sección CIIU principal</t>
-  </si>
-  <si>
-    <t xml:space="preserve">empresas (2022)</t>
   </si>
   <si>
     <t xml:space="preserve">Empresas grandes en la sección</t>
@@ -2989,7 +3007,7 @@
         <v>10</v>
       </c>
       <c r="D93" t="n">
-        <v>592.485477269945</v>
+        <v>4.76691935569091</v>
       </c>
       <c r="E93" t="s">
         <v>23</v>
@@ -3015,7 +3033,7 @@
         <v>14</v>
       </c>
       <c r="D94" t="n">
-        <v>592.485477269945</v>
+        <v>823.433652670573</v>
       </c>
       <c r="E94" t="s">
         <v>23</v>
@@ -3041,7 +3059,7 @@
         <v>15</v>
       </c>
       <c r="D95" t="n">
-        <v>592.485477269945</v>
+        <v>50.3145110316966</v>
       </c>
       <c r="E95" t="s">
         <v>23</v>
@@ -3067,7 +3085,7 @@
         <v>16</v>
       </c>
       <c r="D96" t="n">
-        <v>267.736842581218</v>
+        <v>772.308703908543</v>
       </c>
       <c r="E96" t="s">
         <v>23</v>
@@ -3076,7 +3094,7 @@
         <v>2024</v>
       </c>
       <c r="G96" t="s">
-        <v>26</v>
+        <v>44</v>
       </c>
       <c r="H96" t="s">
         <v>45</v>
@@ -3093,7 +3111,7 @@
         <v>17</v>
       </c>
       <c r="D97" t="n">
-        <v>22.1105026662248</v>
+        <v>1228.59043415906</v>
       </c>
       <c r="E97" t="s">
         <v>23</v>
@@ -3102,7 +3120,7 @@
         <v>2024</v>
       </c>
       <c r="G97" t="s">
-        <v>26</v>
+        <v>44</v>
       </c>
       <c r="H97" t="s">
         <v>45</v>
@@ -3119,7 +3137,7 @@
         <v>18</v>
       </c>
       <c r="D98" t="n">
-        <v>184.040642193553</v>
+        <v>5350.69631342304</v>
       </c>
       <c r="E98" t="s">
         <v>23</v>
@@ -3128,7 +3146,7 @@
         <v>2024</v>
       </c>
       <c r="G98" t="s">
-        <v>26</v>
+        <v>44</v>
       </c>
       <c r="H98" t="s">
         <v>45</v>
@@ -3145,7 +3163,7 @@
         <v>19</v>
       </c>
       <c r="D99" t="n">
-        <v>5572.50001709312</v>
+        <v>22615.1612922376</v>
       </c>
       <c r="E99" t="s">
         <v>23</v>
@@ -3154,7 +3172,7 @@
         <v>2024</v>
       </c>
       <c r="G99" t="s">
-        <v>26</v>
+        <v>44</v>
       </c>
       <c r="H99" t="s">
         <v>45</v>
@@ -3171,7 +3189,7 @@
         <v>10</v>
       </c>
       <c r="D100" t="n">
-        <v>1947.785386979</v>
+        <v>3.68149408632382</v>
       </c>
       <c r="E100" t="s">
         <v>23</v>
@@ -3197,7 +3215,7 @@
         <v>14</v>
       </c>
       <c r="D101" t="n">
-        <v>1947.785386979</v>
+        <v>510.923966855039</v>
       </c>
       <c r="E101" t="s">
         <v>23</v>
@@ -3223,7 +3241,7 @@
         <v>15</v>
       </c>
       <c r="D102" t="n">
-        <v>1947.785386979</v>
+        <v>47.1312383767634</v>
       </c>
       <c r="E102" t="s">
         <v>23</v>
@@ -3249,7 +3267,7 @@
         <v>16</v>
       </c>
       <c r="D103" t="n">
-        <v>2170.73099106753</v>
+        <v>714.934334045153</v>
       </c>
       <c r="E103" t="s">
         <v>23</v>
@@ -3258,7 +3276,7 @@
         <v>2024</v>
       </c>
       <c r="G103" t="s">
-        <v>26</v>
+        <v>44</v>
       </c>
       <c r="H103" t="s">
         <v>45</v>
@@ -3275,7 +3293,7 @@
         <v>17</v>
       </c>
       <c r="D104" t="n">
-        <v>67.3374746397605</v>
+        <v>1000.10818172891</v>
       </c>
       <c r="E104" t="s">
         <v>23</v>
@@ -3284,7 +3302,7 @@
         <v>2024</v>
       </c>
       <c r="G104" t="s">
-        <v>26</v>
+        <v>44</v>
       </c>
       <c r="H104" t="s">
         <v>45</v>
@@ -3301,7 +3319,7 @@
         <v>18</v>
       </c>
       <c r="D105" t="n">
-        <v>1965.67646554552</v>
+        <v>2209.8822924925</v>
       </c>
       <c r="E105" t="s">
         <v>23</v>
@@ -3310,7 +3328,7 @@
         <v>2024</v>
       </c>
       <c r="G105" t="s">
-        <v>26</v>
+        <v>44</v>
       </c>
       <c r="H105" t="s">
         <v>45</v>
@@ -3327,7 +3345,7 @@
         <v>19</v>
       </c>
       <c r="D106" t="n">
-        <v>60468.8554363435</v>
+        <v>18986.4610050005</v>
       </c>
       <c r="E106" t="s">
         <v>23</v>
@@ -3336,7 +3354,7 @@
         <v>2024</v>
       </c>
       <c r="G106" t="s">
-        <v>26</v>
+        <v>44</v>
       </c>
       <c r="H106" t="s">
         <v>45</v>
@@ -3344,22 +3362,22 @@
     </row>
     <row r="107">
       <c r="A107" t="s">
+        <v>42</v>
+      </c>
+      <c r="B107" t="s">
         <v>47</v>
-      </c>
-      <c r="B107" t="s">
-        <v>48</v>
       </c>
       <c r="C107" t="s">
         <v>10</v>
       </c>
       <c r="D107" t="n">
-        <v>188</v>
+        <v>3.68149408632382</v>
       </c>
       <c r="E107" t="s">
-        <v>49</v>
+        <v>23</v>
       </c>
       <c r="F107" t="n">
-        <v>2022</v>
+        <v>2024</v>
       </c>
       <c r="G107" t="s">
         <v>44</v>
@@ -3370,22 +3388,22 @@
     </row>
     <row r="108">
       <c r="A108" t="s">
+        <v>42</v>
+      </c>
+      <c r="B108" t="s">
         <v>47</v>
-      </c>
-      <c r="B108" t="s">
-        <v>48</v>
       </c>
       <c r="C108" t="s">
         <v>14</v>
       </c>
       <c r="D108" t="n">
-        <v>184</v>
+        <v>510.923966855039</v>
       </c>
       <c r="E108" t="s">
-        <v>49</v>
+        <v>23</v>
       </c>
       <c r="F108" t="n">
-        <v>2022</v>
+        <v>2024</v>
       </c>
       <c r="G108" t="s">
         <v>44</v>
@@ -3396,22 +3414,22 @@
     </row>
     <row r="109">
       <c r="A109" t="s">
+        <v>42</v>
+      </c>
+      <c r="B109" t="s">
         <v>47</v>
-      </c>
-      <c r="B109" t="s">
-        <v>48</v>
       </c>
       <c r="C109" t="s">
         <v>15</v>
       </c>
       <c r="D109" t="n">
-        <v>188</v>
+        <v>47.1312383767634</v>
       </c>
       <c r="E109" t="s">
-        <v>49</v>
+        <v>23</v>
       </c>
       <c r="F109" t="n">
-        <v>2022</v>
+        <v>2024</v>
       </c>
       <c r="G109" t="s">
         <v>44</v>
@@ -3422,22 +3440,22 @@
     </row>
     <row r="110">
       <c r="A110" t="s">
+        <v>42</v>
+      </c>
+      <c r="B110" t="s">
         <v>47</v>
-      </c>
-      <c r="B110" t="s">
-        <v>48</v>
       </c>
       <c r="C110" t="s">
         <v>16</v>
       </c>
       <c r="D110" t="n">
-        <v>5123</v>
+        <v>772.308703908543</v>
       </c>
       <c r="E110" t="s">
-        <v>49</v>
+        <v>23</v>
       </c>
       <c r="F110" t="n">
-        <v>2022</v>
+        <v>2024</v>
       </c>
       <c r="G110" t="s">
         <v>44</v>
@@ -3448,22 +3466,22 @@
     </row>
     <row r="111">
       <c r="A111" t="s">
+        <v>42</v>
+      </c>
+      <c r="B111" t="s">
         <v>47</v>
-      </c>
-      <c r="B111" t="s">
-        <v>48</v>
       </c>
       <c r="C111" t="s">
         <v>17</v>
       </c>
       <c r="D111" t="n">
-        <v>942</v>
+        <v>1000.10818172891</v>
       </c>
       <c r="E111" t="s">
-        <v>49</v>
+        <v>23</v>
       </c>
       <c r="F111" t="n">
-        <v>2022</v>
+        <v>2024</v>
       </c>
       <c r="G111" t="s">
         <v>44</v>
@@ -3474,22 +3492,22 @@
     </row>
     <row r="112">
       <c r="A112" t="s">
+        <v>42</v>
+      </c>
+      <c r="B112" t="s">
         <v>47</v>
-      </c>
-      <c r="B112" t="s">
-        <v>48</v>
       </c>
       <c r="C112" t="s">
         <v>18</v>
       </c>
       <c r="D112" t="n">
-        <v>2567</v>
+        <v>2209.8822924925</v>
       </c>
       <c r="E112" t="s">
-        <v>49</v>
+        <v>23</v>
       </c>
       <c r="F112" t="n">
-        <v>2022</v>
+        <v>2024</v>
       </c>
       <c r="G112" t="s">
         <v>44</v>
@@ -3500,22 +3518,22 @@
     </row>
     <row r="113">
       <c r="A113" t="s">
+        <v>42</v>
+      </c>
+      <c r="B113" t="s">
         <v>47</v>
       </c>
-      <c r="B113" t="s">
-        <v>50</v>
-      </c>
       <c r="C113" t="s">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="D113" t="n">
-        <v>12.2340425531915</v>
+        <v>22615.1612922376</v>
       </c>
       <c r="E113" t="s">
-        <v>51</v>
+        <v>23</v>
       </c>
       <c r="F113" t="n">
-        <v>2022</v>
+        <v>2024</v>
       </c>
       <c r="G113" t="s">
         <v>44</v>
@@ -3526,22 +3544,22 @@
     </row>
     <row r="114">
       <c r="A114" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="B114" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C114" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="D114" t="n">
-        <v>38.5869565217391</v>
+        <v>592.485477269945</v>
       </c>
       <c r="E114" t="s">
-        <v>51</v>
+        <v>23</v>
       </c>
       <c r="F114" t="n">
-        <v>2022</v>
+        <v>2024</v>
       </c>
       <c r="G114" t="s">
         <v>44</v>
@@ -3552,22 +3570,22 @@
     </row>
     <row r="115">
       <c r="A115" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="B115" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C115" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D115" t="n">
-        <v>12.2340425531915</v>
+        <v>592.485477269945</v>
       </c>
       <c r="E115" t="s">
-        <v>51</v>
+        <v>23</v>
       </c>
       <c r="F115" t="n">
-        <v>2022</v>
+        <v>2024</v>
       </c>
       <c r="G115" t="s">
         <v>44</v>
@@ -3578,22 +3596,22 @@
     </row>
     <row r="116">
       <c r="A116" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="B116" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C116" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D116" t="n">
-        <v>5.4850673433535</v>
+        <v>592.485477269945</v>
       </c>
       <c r="E116" t="s">
-        <v>51</v>
+        <v>23</v>
       </c>
       <c r="F116" t="n">
-        <v>2022</v>
+        <v>2024</v>
       </c>
       <c r="G116" t="s">
         <v>44</v>
@@ -3604,25 +3622,25 @@
     </row>
     <row r="117">
       <c r="A117" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="B117" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C117" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D117" t="n">
-        <v>5.73248407643312</v>
+        <v>267.736842581218</v>
       </c>
       <c r="E117" t="s">
-        <v>51</v>
+        <v>23</v>
       </c>
       <c r="F117" t="n">
-        <v>2022</v>
+        <v>2024</v>
       </c>
       <c r="G117" t="s">
-        <v>44</v>
+        <v>26</v>
       </c>
       <c r="H117" t="s">
         <v>45</v>
@@ -3630,25 +3648,25 @@
     </row>
     <row r="118">
       <c r="A118" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="B118" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C118" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D118" t="n">
-        <v>8.10284378652123</v>
+        <v>22.1105026662248</v>
       </c>
       <c r="E118" t="s">
-        <v>51</v>
+        <v>23</v>
       </c>
       <c r="F118" t="n">
-        <v>2022</v>
+        <v>2024</v>
       </c>
       <c r="G118" t="s">
-        <v>44</v>
+        <v>26</v>
       </c>
       <c r="H118" t="s">
         <v>45</v>
@@ -3656,1380 +3674,1380 @@
     </row>
     <row r="119">
       <c r="A119" t="s">
-        <v>52</v>
+        <v>42</v>
       </c>
       <c r="B119" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="C119" t="s">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="D119" t="n">
-        <v>1897.79224114914</v>
+        <v>184.040642193553</v>
       </c>
       <c r="E119" t="s">
-        <v>54</v>
+        <v>23</v>
       </c>
       <c r="F119" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="G119" t="s">
         <v>26</v>
       </c>
       <c r="H119" t="s">
-        <v>55</v>
+        <v>45</v>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="s">
-        <v>52</v>
+        <v>42</v>
       </c>
       <c r="B120" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="C120" t="s">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="D120" t="n">
-        <v>4163.08133121177</v>
+        <v>5572.50001709312</v>
       </c>
       <c r="E120" t="s">
-        <v>54</v>
+        <v>23</v>
       </c>
       <c r="F120" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="G120" t="s">
         <v>26</v>
       </c>
       <c r="H120" t="s">
-        <v>55</v>
+        <v>45</v>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="s">
-        <v>52</v>
+        <v>42</v>
       </c>
       <c r="B121" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="C121" t="s">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="D121" t="n">
-        <v>2327.78580311458</v>
+        <v>1947.785386979</v>
       </c>
       <c r="E121" t="s">
-        <v>54</v>
+        <v>23</v>
       </c>
       <c r="F121" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="G121" t="s">
-        <v>26</v>
+        <v>44</v>
       </c>
       <c r="H121" t="s">
-        <v>55</v>
+        <v>45</v>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="s">
-        <v>52</v>
+        <v>42</v>
       </c>
       <c r="B122" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="C122" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D122" t="n">
-        <v>3789.73322355154</v>
+        <v>1947.785386979</v>
       </c>
       <c r="E122" t="s">
-        <v>54</v>
+        <v>23</v>
       </c>
       <c r="F122" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="G122" t="s">
-        <v>26</v>
+        <v>44</v>
       </c>
       <c r="H122" t="s">
-        <v>55</v>
+        <v>45</v>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="s">
-        <v>52</v>
+        <v>42</v>
       </c>
       <c r="B123" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="C123" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="D123" t="n">
-        <v>7600.79697287293</v>
+        <v>1947.785386979</v>
       </c>
       <c r="E123" t="s">
-        <v>54</v>
+        <v>23</v>
       </c>
       <c r="F123" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="G123" t="s">
-        <v>26</v>
+        <v>44</v>
       </c>
       <c r="H123" t="s">
-        <v>55</v>
+        <v>45</v>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="s">
-        <v>52</v>
+        <v>42</v>
       </c>
       <c r="B124" t="s">
-        <v>56</v>
+        <v>49</v>
       </c>
       <c r="C124" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="D124" t="n">
-        <v>22.4919511076553</v>
+        <v>2170.73099106753</v>
       </c>
       <c r="E124" t="s">
-        <v>57</v>
+        <v>23</v>
       </c>
       <c r="F124" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="G124" t="s">
         <v>26</v>
       </c>
       <c r="H124" t="s">
-        <v>55</v>
+        <v>45</v>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="s">
-        <v>52</v>
+        <v>42</v>
       </c>
       <c r="B125" t="s">
-        <v>56</v>
+        <v>49</v>
       </c>
       <c r="C125" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="D125" t="n">
-        <v>2.45503983060696</v>
+        <v>67.3374746397605</v>
       </c>
       <c r="E125" t="s">
-        <v>57</v>
+        <v>23</v>
       </c>
       <c r="F125" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="G125" t="s">
         <v>26</v>
       </c>
       <c r="H125" t="s">
-        <v>55</v>
+        <v>45</v>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="s">
-        <v>52</v>
+        <v>42</v>
       </c>
       <c r="B126" t="s">
-        <v>56</v>
+        <v>49</v>
       </c>
       <c r="C126" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="D126" t="n">
-        <v>1.01347910248753</v>
+        <v>1965.67646554552</v>
       </c>
       <c r="E126" t="s">
-        <v>57</v>
+        <v>23</v>
       </c>
       <c r="F126" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="G126" t="s">
         <v>26</v>
       </c>
       <c r="H126" t="s">
-        <v>55</v>
+        <v>45</v>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="s">
-        <v>52</v>
+        <v>42</v>
       </c>
       <c r="B127" t="s">
-        <v>56</v>
+        <v>49</v>
       </c>
       <c r="C127" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="D127" t="n">
-        <v>0.960608594795822</v>
+        <v>60468.8554363435</v>
       </c>
       <c r="E127" t="s">
-        <v>57</v>
+        <v>23</v>
       </c>
       <c r="F127" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="G127" t="s">
         <v>26</v>
       </c>
       <c r="H127" t="s">
-        <v>55</v>
+        <v>45</v>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="s">
-        <v>52</v>
+        <v>42</v>
       </c>
       <c r="B128" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="C128" t="s">
         <v>10</v>
       </c>
       <c r="D128" t="n">
-        <v>9.5948938365266</v>
+        <v>4.69706788056383</v>
       </c>
       <c r="E128" t="s">
-        <v>21</v>
+        <v>51</v>
       </c>
       <c r="F128" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="G128" t="s">
-        <v>26</v>
+        <v>44</v>
       </c>
       <c r="H128" t="s">
-        <v>55</v>
+        <v>45</v>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="s">
-        <v>52</v>
+        <v>42</v>
       </c>
       <c r="B129" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="C129" t="s">
         <v>14</v>
       </c>
       <c r="D129" t="n">
-        <v>21.0477851788539</v>
+        <v>27.7928105174365</v>
       </c>
       <c r="E129" t="s">
-        <v>21</v>
+        <v>51</v>
       </c>
       <c r="F129" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="G129" t="s">
-        <v>26</v>
+        <v>44</v>
       </c>
       <c r="H129" t="s">
-        <v>55</v>
+        <v>45</v>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="s">
-        <v>52</v>
+        <v>42</v>
       </c>
       <c r="B130" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="C130" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D130" t="n">
-        <v>11.7688634038962</v>
+        <v>26.9338785542736</v>
       </c>
       <c r="E130" t="s">
-        <v>21</v>
+        <v>51</v>
       </c>
       <c r="F130" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="G130" t="s">
-        <v>26</v>
+        <v>44</v>
       </c>
       <c r="H130" t="s">
-        <v>55</v>
+        <v>45</v>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="s">
-        <v>52</v>
+        <v>42</v>
       </c>
       <c r="B131" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="C131" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D131" t="n">
-        <v>19.16020476863</v>
+        <v>33.4296982614687</v>
       </c>
       <c r="E131" t="s">
-        <v>21</v>
+        <v>51</v>
       </c>
       <c r="F131" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="G131" t="s">
-        <v>26</v>
+        <v>44</v>
       </c>
       <c r="H131" t="s">
-        <v>55</v>
+        <v>45</v>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="s">
-        <v>52</v>
+        <v>42</v>
       </c>
       <c r="B132" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="C132" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="D132" t="n">
-        <v>38.4282528120934</v>
+        <v>24.8653622297221</v>
       </c>
       <c r="E132" t="s">
-        <v>21</v>
+        <v>51</v>
       </c>
       <c r="F132" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="G132" t="s">
-        <v>26</v>
+        <v>44</v>
       </c>
       <c r="H132" t="s">
-        <v>55</v>
+        <v>45</v>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="s">
-        <v>59</v>
+        <v>42</v>
       </c>
       <c r="B133" t="s">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="C133" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="D133" t="n">
-        <v>1772.04693496869</v>
+        <v>14.2032288156637</v>
       </c>
       <c r="E133" t="s">
-        <v>61</v>
+        <v>51</v>
       </c>
       <c r="F133" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="G133" t="s">
-        <v>26</v>
+        <v>44</v>
       </c>
       <c r="H133" t="s">
-        <v>62</v>
+        <v>45</v>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="s">
-        <v>59</v>
+        <v>42</v>
       </c>
       <c r="B134" t="s">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="C134" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="D134" t="n">
-        <v>4708.1023828052</v>
+        <v>36.4974073158468</v>
       </c>
       <c r="E134" t="s">
-        <v>61</v>
+        <v>51</v>
       </c>
       <c r="F134" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="G134" t="s">
-        <v>26</v>
+        <v>44</v>
       </c>
       <c r="H134" t="s">
-        <v>62</v>
+        <v>45</v>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="s">
-        <v>59</v>
+        <v>52</v>
       </c>
       <c r="B135" t="s">
-        <v>60</v>
+        <v>53</v>
       </c>
       <c r="C135" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="D135" t="n">
-        <v>255.5815730824</v>
+        <v>188</v>
       </c>
       <c r="E135" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="F135" t="n">
-        <v>2023</v>
+        <v>2022</v>
       </c>
       <c r="G135" t="s">
-        <v>26</v>
+        <v>44</v>
       </c>
       <c r="H135" t="s">
-        <v>62</v>
+        <v>55</v>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="s">
-        <v>59</v>
+        <v>52</v>
       </c>
       <c r="B136" t="s">
-        <v>60</v>
+        <v>53</v>
       </c>
       <c r="C136" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="D136" t="n">
-        <v>23625.8901555541</v>
+        <v>184</v>
       </c>
       <c r="E136" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="F136" t="n">
-        <v>2023</v>
+        <v>2022</v>
       </c>
       <c r="G136" t="s">
-        <v>26</v>
+        <v>44</v>
       </c>
       <c r="H136" t="s">
-        <v>62</v>
+        <v>55</v>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="s">
-        <v>59</v>
+        <v>52</v>
       </c>
       <c r="B137" t="s">
-        <v>63</v>
+        <v>53</v>
       </c>
       <c r="C137" t="s">
         <v>15</v>
       </c>
       <c r="D137" t="n">
-        <v>759.10000005414</v>
+        <v>188</v>
       </c>
       <c r="E137" t="s">
-        <v>64</v>
+        <v>54</v>
       </c>
       <c r="F137" t="n">
         <v>2022</v>
       </c>
       <c r="G137" t="s">
-        <v>26</v>
+        <v>44</v>
       </c>
       <c r="H137" t="s">
-        <v>62</v>
+        <v>55</v>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="s">
-        <v>59</v>
+        <v>52</v>
       </c>
       <c r="B138" t="s">
-        <v>63</v>
+        <v>53</v>
       </c>
       <c r="C138" t="s">
         <v>16</v>
       </c>
       <c r="D138" t="n">
-        <v>6.200000003736</v>
+        <v>5123</v>
       </c>
       <c r="E138" t="s">
-        <v>64</v>
+        <v>54</v>
       </c>
       <c r="F138" t="n">
         <v>2022</v>
       </c>
       <c r="G138" t="s">
-        <v>26</v>
+        <v>44</v>
       </c>
       <c r="H138" t="s">
-        <v>62</v>
+        <v>55</v>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="s">
-        <v>59</v>
+        <v>52</v>
       </c>
       <c r="B139" t="s">
-        <v>63</v>
+        <v>53</v>
       </c>
       <c r="C139" t="s">
         <v>17</v>
       </c>
       <c r="D139" t="n">
-        <v>446.09999999058</v>
+        <v>942</v>
       </c>
       <c r="E139" t="s">
-        <v>64</v>
+        <v>54</v>
       </c>
       <c r="F139" t="n">
         <v>2022</v>
       </c>
       <c r="G139" t="s">
-        <v>26</v>
+        <v>44</v>
       </c>
       <c r="H139" t="s">
-        <v>62</v>
+        <v>55</v>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="s">
-        <v>59</v>
+        <v>52</v>
       </c>
       <c r="B140" t="s">
-        <v>65</v>
+        <v>53</v>
       </c>
       <c r="C140" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="D140" t="n">
-        <v>1.04500620116081</v>
+        <v>2567</v>
       </c>
       <c r="E140" t="s">
-        <v>66</v>
+        <v>54</v>
       </c>
       <c r="F140" t="n">
-        <v>2023</v>
+        <v>2022</v>
       </c>
       <c r="G140" t="s">
-        <v>26</v>
+        <v>44</v>
       </c>
       <c r="H140" t="s">
-        <v>62</v>
+        <v>55</v>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="s">
-        <v>59</v>
+        <v>52</v>
       </c>
       <c r="B141" t="s">
-        <v>65</v>
+        <v>56</v>
       </c>
       <c r="C141" t="s">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="D141" t="n">
-        <v>2.04982922868611</v>
+        <v>12.2340425531915</v>
       </c>
       <c r="E141" t="s">
-        <v>66</v>
+        <v>57</v>
       </c>
       <c r="F141" t="n">
-        <v>2023</v>
+        <v>2022</v>
       </c>
       <c r="G141" t="s">
-        <v>26</v>
+        <v>44</v>
       </c>
       <c r="H141" t="s">
-        <v>62</v>
+        <v>55</v>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="s">
-        <v>59</v>
+        <v>52</v>
       </c>
       <c r="B142" t="s">
-        <v>65</v>
+        <v>56</v>
       </c>
       <c r="C142" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D142" t="n">
-        <v>0.0647839415842331</v>
+        <v>38.5869565217391</v>
       </c>
       <c r="E142" t="s">
-        <v>66</v>
+        <v>57</v>
       </c>
       <c r="F142" t="n">
-        <v>2023</v>
+        <v>2022</v>
       </c>
       <c r="G142" t="s">
-        <v>26</v>
+        <v>44</v>
       </c>
       <c r="H142" t="s">
-        <v>62</v>
+        <v>55</v>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="s">
-        <v>59</v>
+        <v>52</v>
       </c>
       <c r="B143" t="s">
-        <v>65</v>
+        <v>56</v>
       </c>
       <c r="C143" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="D143" t="n">
-        <v>0.39855220768945</v>
+        <v>12.2340425531915</v>
       </c>
       <c r="E143" t="s">
-        <v>66</v>
+        <v>57</v>
       </c>
       <c r="F143" t="n">
-        <v>2023</v>
+        <v>2022</v>
       </c>
       <c r="G143" t="s">
-        <v>26</v>
+        <v>44</v>
       </c>
       <c r="H143" t="s">
-        <v>62</v>
+        <v>55</v>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="s">
-        <v>67</v>
+        <v>52</v>
       </c>
       <c r="B144" t="s">
-        <v>68</v>
+        <v>56</v>
       </c>
       <c r="C144" t="s">
         <v>16</v>
       </c>
       <c r="D144" t="n">
-        <v>882966.0616672</v>
+        <v>5.4850673433535</v>
       </c>
       <c r="E144" t="s">
-        <v>69</v>
+        <v>57</v>
       </c>
       <c r="F144" t="n">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="G144" t="s">
         <v>44</v>
       </c>
       <c r="H144" t="s">
-        <v>62</v>
+        <v>55</v>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="s">
-        <v>67</v>
+        <v>52</v>
       </c>
       <c r="B145" t="s">
-        <v>70</v>
+        <v>56</v>
       </c>
       <c r="C145" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D145" t="n">
-        <v>1072852</v>
+        <v>5.73248407643312</v>
       </c>
       <c r="E145" t="s">
-        <v>69</v>
+        <v>57</v>
       </c>
       <c r="F145" t="n">
-        <v>2015</v>
+        <v>2022</v>
       </c>
       <c r="G145" t="s">
         <v>44</v>
       </c>
       <c r="H145" t="s">
-        <v>62</v>
+        <v>55</v>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="s">
-        <v>67</v>
+        <v>52</v>
       </c>
       <c r="B146" t="s">
-        <v>71</v>
+        <v>56</v>
       </c>
       <c r="C146" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D146" t="n">
-        <v>650399.1079245</v>
+        <v>8.10284378652123</v>
       </c>
       <c r="E146" t="s">
-        <v>69</v>
+        <v>57</v>
       </c>
       <c r="F146" t="n">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="G146" t="s">
         <v>44</v>
       </c>
       <c r="H146" t="s">
-        <v>62</v>
+        <v>55</v>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="s">
-        <v>67</v>
+        <v>58</v>
       </c>
       <c r="B147" t="s">
-        <v>72</v>
+        <v>59</v>
       </c>
       <c r="C147" t="s">
         <v>10</v>
       </c>
       <c r="D147" t="n">
-        <v>1970906.38765</v>
+        <v>1897.79224114914</v>
       </c>
       <c r="E147" t="s">
-        <v>69</v>
+        <v>60</v>
       </c>
       <c r="F147" t="n">
-        <v>2021</v>
+        <v>2023</v>
       </c>
       <c r="G147" t="s">
-        <v>44</v>
+        <v>26</v>
       </c>
       <c r="H147" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="s">
-        <v>73</v>
+        <v>58</v>
       </c>
       <c r="B148" t="s">
-        <v>74</v>
+        <v>59</v>
       </c>
       <c r="C148" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="D148" t="n">
-        <v>1.00972599678899</v>
+        <v>4163.08133121177</v>
       </c>
       <c r="E148" t="s">
-        <v>75</v>
+        <v>60</v>
       </c>
       <c r="F148" t="n">
-        <v>2018</v>
+        <v>2023</v>
       </c>
       <c r="G148" t="s">
         <v>26</v>
       </c>
       <c r="H148" t="s">
-        <v>76</v>
+        <v>61</v>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="s">
-        <v>73</v>
+        <v>58</v>
       </c>
       <c r="B149" t="s">
-        <v>74</v>
+        <v>59</v>
       </c>
       <c r="C149" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="D149" t="n">
-        <v>1.38463301489268</v>
+        <v>2327.78580311458</v>
       </c>
       <c r="E149" t="s">
-        <v>75</v>
+        <v>60</v>
       </c>
       <c r="F149" t="n">
-        <v>2018</v>
+        <v>2023</v>
       </c>
       <c r="G149" t="s">
         <v>26</v>
       </c>
       <c r="H149" t="s">
-        <v>76</v>
+        <v>61</v>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="s">
-        <v>73</v>
+        <v>58</v>
       </c>
       <c r="B150" t="s">
-        <v>74</v>
+        <v>59</v>
       </c>
       <c r="C150" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="D150" t="n">
-        <v>1.01159962166824</v>
+        <v>3789.73322355154</v>
       </c>
       <c r="E150" t="s">
-        <v>75</v>
+        <v>60</v>
       </c>
       <c r="F150" t="n">
-        <v>2018</v>
+        <v>2023</v>
       </c>
       <c r="G150" t="s">
         <v>26</v>
       </c>
       <c r="H150" t="s">
-        <v>76</v>
+        <v>61</v>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="s">
-        <v>73</v>
+        <v>58</v>
       </c>
       <c r="B151" t="s">
-        <v>74</v>
+        <v>59</v>
       </c>
       <c r="C151" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="D151" t="n">
-        <v>1.34113695951916</v>
+        <v>7600.79697287293</v>
       </c>
       <c r="E151" t="s">
-        <v>75</v>
+        <v>60</v>
       </c>
       <c r="F151" t="n">
-        <v>2018</v>
+        <v>2023</v>
       </c>
       <c r="G151" t="s">
         <v>26</v>
       </c>
       <c r="H151" t="s">
-        <v>76</v>
+        <v>61</v>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="s">
-        <v>73</v>
+        <v>58</v>
       </c>
       <c r="B152" t="s">
-        <v>74</v>
+        <v>62</v>
       </c>
       <c r="C152" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="D152" t="n">
-        <v>1.51107677264798</v>
+        <v>22.4919511076553</v>
       </c>
       <c r="E152" t="s">
-        <v>75</v>
+        <v>63</v>
       </c>
       <c r="F152" t="n">
-        <v>2018</v>
+        <v>2023</v>
       </c>
       <c r="G152" t="s">
         <v>26</v>
       </c>
       <c r="H152" t="s">
-        <v>76</v>
+        <v>61</v>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="s">
-        <v>73</v>
+        <v>58</v>
       </c>
       <c r="B153" t="s">
-        <v>74</v>
+        <v>62</v>
       </c>
       <c r="C153" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="D153" t="n">
-        <v>1.10028979595841</v>
+        <v>2.45503983060696</v>
       </c>
       <c r="E153" t="s">
-        <v>75</v>
+        <v>63</v>
       </c>
       <c r="F153" t="n">
-        <v>2018</v>
+        <v>2023</v>
       </c>
       <c r="G153" t="s">
         <v>26</v>
       </c>
       <c r="H153" t="s">
-        <v>76</v>
+        <v>61</v>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="s">
-        <v>73</v>
+        <v>58</v>
       </c>
       <c r="B154" t="s">
-        <v>74</v>
+        <v>62</v>
       </c>
       <c r="C154" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D154" t="n">
-        <v>2.67558022226578</v>
+        <v>1.01347910248753</v>
       </c>
       <c r="E154" t="s">
-        <v>75</v>
+        <v>63</v>
       </c>
       <c r="F154" t="n">
-        <v>2018</v>
+        <v>2023</v>
       </c>
       <c r="G154" t="s">
         <v>26</v>
       </c>
       <c r="H154" t="s">
-        <v>76</v>
+        <v>61</v>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="s">
-        <v>73</v>
+        <v>58</v>
       </c>
       <c r="B155" t="s">
-        <v>77</v>
+        <v>62</v>
       </c>
       <c r="C155" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="D155" t="n">
-        <v>1.35461522604007</v>
+        <v>0.960608594795822</v>
       </c>
       <c r="E155" t="s">
-        <v>75</v>
+        <v>63</v>
       </c>
       <c r="F155" t="n">
-        <v>2018</v>
+        <v>2023</v>
       </c>
       <c r="G155" t="s">
         <v>26</v>
       </c>
       <c r="H155" t="s">
-        <v>76</v>
+        <v>61</v>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="s">
-        <v>73</v>
+        <v>58</v>
       </c>
       <c r="B156" t="s">
-        <v>77</v>
+        <v>64</v>
       </c>
       <c r="C156" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="D156" t="n">
-        <v>1.33052676362134</v>
+        <v>9.5948938365266</v>
       </c>
       <c r="E156" t="s">
-        <v>75</v>
+        <v>21</v>
       </c>
       <c r="F156" t="n">
-        <v>2018</v>
+        <v>2023</v>
       </c>
       <c r="G156" t="s">
         <v>26</v>
       </c>
       <c r="H156" t="s">
-        <v>76</v>
+        <v>61</v>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="s">
-        <v>73</v>
+        <v>58</v>
       </c>
       <c r="B157" t="s">
-        <v>77</v>
+        <v>64</v>
       </c>
       <c r="C157" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D157" t="n">
-        <v>1.44639724826724</v>
+        <v>21.0477851788539</v>
       </c>
       <c r="E157" t="s">
-        <v>75</v>
+        <v>21</v>
       </c>
       <c r="F157" t="n">
-        <v>2018</v>
+        <v>2023</v>
       </c>
       <c r="G157" t="s">
         <v>26</v>
       </c>
       <c r="H157" t="s">
-        <v>76</v>
+        <v>61</v>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="s">
-        <v>73</v>
+        <v>58</v>
       </c>
       <c r="B158" t="s">
-        <v>77</v>
+        <v>64</v>
       </c>
       <c r="C158" t="s">
         <v>16</v>
       </c>
       <c r="D158" t="n">
-        <v>1.50003805694812</v>
+        <v>11.7688634038962</v>
       </c>
       <c r="E158" t="s">
-        <v>75</v>
+        <v>21</v>
       </c>
       <c r="F158" t="n">
-        <v>2018</v>
+        <v>2023</v>
       </c>
       <c r="G158" t="s">
         <v>26</v>
       </c>
       <c r="H158" t="s">
-        <v>76</v>
+        <v>61</v>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="s">
-        <v>73</v>
+        <v>58</v>
       </c>
       <c r="B159" t="s">
-        <v>77</v>
+        <v>64</v>
       </c>
       <c r="C159" t="s">
         <v>17</v>
       </c>
       <c r="D159" t="n">
-        <v>1.67606087093891</v>
+        <v>19.16020476863</v>
       </c>
       <c r="E159" t="s">
-        <v>75</v>
+        <v>21</v>
       </c>
       <c r="F159" t="n">
-        <v>2018</v>
+        <v>2023</v>
       </c>
       <c r="G159" t="s">
         <v>26</v>
       </c>
       <c r="H159" t="s">
-        <v>76</v>
+        <v>61</v>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="s">
-        <v>73</v>
+        <v>58</v>
       </c>
       <c r="B160" t="s">
-        <v>77</v>
+        <v>64</v>
       </c>
       <c r="C160" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D160" t="n">
-        <v>1.40536722167565</v>
+        <v>38.4282528120934</v>
       </c>
       <c r="E160" t="s">
-        <v>75</v>
+        <v>21</v>
       </c>
       <c r="F160" t="n">
-        <v>2018</v>
+        <v>2023</v>
       </c>
       <c r="G160" t="s">
         <v>26</v>
       </c>
       <c r="H160" t="s">
-        <v>76</v>
+        <v>61</v>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="s">
-        <v>73</v>
+        <v>65</v>
       </c>
       <c r="B161" t="s">
-        <v>77</v>
+        <v>66</v>
       </c>
       <c r="C161" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="D161" t="n">
-        <v>1.32103699624993</v>
+        <v>1772.04693496869</v>
       </c>
       <c r="E161" t="s">
-        <v>75</v>
+        <v>67</v>
       </c>
       <c r="F161" t="n">
-        <v>2018</v>
+        <v>2023</v>
       </c>
       <c r="G161" t="s">
         <v>26</v>
       </c>
       <c r="H161" t="s">
-        <v>76</v>
+        <v>68</v>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="s">
-        <v>73</v>
+        <v>65</v>
       </c>
       <c r="B162" t="s">
-        <v>78</v>
+        <v>66</v>
       </c>
       <c r="C162" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="D162" t="n">
-        <v>41.2818689801426</v>
+        <v>4708.1023828052</v>
       </c>
       <c r="E162" t="s">
-        <v>79</v>
+        <v>67</v>
       </c>
       <c r="F162" t="n">
-        <v>2018</v>
+        <v>2023</v>
       </c>
       <c r="G162" t="s">
         <v>26</v>
       </c>
       <c r="H162" t="s">
-        <v>76</v>
+        <v>68</v>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="s">
-        <v>73</v>
+        <v>65</v>
       </c>
       <c r="B163" t="s">
-        <v>78</v>
+        <v>66</v>
       </c>
       <c r="C163" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="D163" t="n">
-        <v>6.58456873124472</v>
+        <v>255.5815730824</v>
       </c>
       <c r="E163" t="s">
-        <v>79</v>
+        <v>67</v>
       </c>
       <c r="F163" t="n">
-        <v>2018</v>
+        <v>2023</v>
       </c>
       <c r="G163" t="s">
         <v>26</v>
       </c>
       <c r="H163" t="s">
-        <v>76</v>
+        <v>68</v>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="s">
-        <v>73</v>
+        <v>65</v>
       </c>
       <c r="B164" t="s">
-        <v>78</v>
+        <v>66</v>
       </c>
       <c r="C164" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="D164" t="n">
-        <v>17.2338509998643</v>
+        <v>23625.8901555541</v>
       </c>
       <c r="E164" t="s">
-        <v>79</v>
+        <v>67</v>
       </c>
       <c r="F164" t="n">
-        <v>2018</v>
+        <v>2023</v>
       </c>
       <c r="G164" t="s">
         <v>26</v>
       </c>
       <c r="H164" t="s">
-        <v>76</v>
+        <v>68</v>
       </c>
     </row>
     <row r="165">
       <c r="A165" t="s">
-        <v>73</v>
+        <v>65</v>
       </c>
       <c r="B165" t="s">
-        <v>78</v>
+        <v>69</v>
       </c>
       <c r="C165" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D165" t="n">
-        <v>27.3242498786245</v>
+        <v>759.10000005414</v>
       </c>
       <c r="E165" t="s">
-        <v>79</v>
+        <v>70</v>
       </c>
       <c r="F165" t="n">
-        <v>2018</v>
+        <v>2022</v>
       </c>
       <c r="G165" t="s">
         <v>26</v>
       </c>
       <c r="H165" t="s">
-        <v>76</v>
+        <v>68</v>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="s">
-        <v>73</v>
+        <v>65</v>
       </c>
       <c r="B166" t="s">
-        <v>78</v>
+        <v>69</v>
       </c>
       <c r="C166" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D166" t="n">
-        <v>78.7763190160058</v>
+        <v>6.200000003736</v>
       </c>
       <c r="E166" t="s">
-        <v>79</v>
+        <v>70</v>
       </c>
       <c r="F166" t="n">
-        <v>2018</v>
+        <v>2022</v>
       </c>
       <c r="G166" t="s">
         <v>26</v>
       </c>
       <c r="H166" t="s">
-        <v>76</v>
+        <v>68</v>
       </c>
     </row>
     <row r="167">
       <c r="A167" t="s">
-        <v>73</v>
+        <v>65</v>
       </c>
       <c r="B167" t="s">
-        <v>78</v>
+        <v>69</v>
       </c>
       <c r="C167" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D167" t="n">
-        <v>16.4076079379625</v>
+        <v>446.09999999058</v>
       </c>
       <c r="E167" t="s">
-        <v>79</v>
+        <v>70</v>
       </c>
       <c r="F167" t="n">
-        <v>2018</v>
+        <v>2022</v>
       </c>
       <c r="G167" t="s">
         <v>26</v>
       </c>
       <c r="H167" t="s">
-        <v>76</v>
+        <v>68</v>
       </c>
     </row>
     <row r="168">
       <c r="A168" t="s">
-        <v>73</v>
+        <v>65</v>
       </c>
       <c r="B168" t="s">
-        <v>78</v>
+        <v>71</v>
       </c>
       <c r="C168" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="D168" t="n">
-        <v>25.3412219653864</v>
+        <v>1.04500620116081</v>
       </c>
       <c r="E168" t="s">
-        <v>79</v>
+        <v>72</v>
       </c>
       <c r="F168" t="n">
-        <v>2018</v>
+        <v>2023</v>
       </c>
       <c r="G168" t="s">
         <v>26</v>
       </c>
       <c r="H168" t="s">
-        <v>76</v>
+        <v>68</v>
       </c>
     </row>
     <row r="169">
       <c r="A169" t="s">
-        <v>73</v>
+        <v>65</v>
       </c>
       <c r="B169" t="s">
-        <v>80</v>
+        <v>71</v>
       </c>
       <c r="C169" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="D169" t="n">
-        <v>0.87377430071436</v>
+        <v>2.04982922868611</v>
       </c>
       <c r="E169" t="s">
-        <v>81</v>
+        <v>72</v>
       </c>
       <c r="F169" t="n">
-        <v>2018</v>
+        <v>2023</v>
       </c>
       <c r="G169" t="s">
         <v>26</v>
       </c>
       <c r="H169" t="s">
-        <v>76</v>
+        <v>68</v>
       </c>
     </row>
     <row r="170">
       <c r="A170" t="s">
-        <v>73</v>
+        <v>65</v>
       </c>
       <c r="B170" t="s">
-        <v>80</v>
+        <v>71</v>
       </c>
       <c r="C170" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="D170" t="n">
-        <v>0.882565776633652</v>
+        <v>0.0647839415842331</v>
       </c>
       <c r="E170" t="s">
-        <v>81</v>
+        <v>72</v>
       </c>
       <c r="F170" t="n">
-        <v>2018</v>
+        <v>2023</v>
       </c>
       <c r="G170" t="s">
         <v>26</v>
       </c>
       <c r="H170" t="s">
-        <v>76</v>
+        <v>68</v>
       </c>
     </row>
     <row r="171">
       <c r="A171" t="s">
-        <v>73</v>
+        <v>65</v>
       </c>
       <c r="B171" t="s">
-        <v>80</v>
+        <v>71</v>
       </c>
       <c r="C171" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="D171" t="n">
-        <v>0.874031286778138</v>
+        <v>0.39855220768945</v>
       </c>
       <c r="E171" t="s">
-        <v>81</v>
+        <v>72</v>
       </c>
       <c r="F171" t="n">
-        <v>2018</v>
+        <v>2023</v>
       </c>
       <c r="G171" t="s">
         <v>26</v>
       </c>
       <c r="H171" t="s">
-        <v>76</v>
+        <v>68</v>
       </c>
     </row>
     <row r="172">
@@ -5037,25 +5055,25 @@
         <v>73</v>
       </c>
       <c r="B172" t="s">
-        <v>80</v>
+        <v>74</v>
       </c>
       <c r="C172" t="s">
         <v>16</v>
       </c>
       <c r="D172" t="n">
-        <v>0.7700582389548</v>
+        <v>882966.0616672</v>
       </c>
       <c r="E172" t="s">
-        <v>81</v>
+        <v>75</v>
       </c>
       <c r="F172" t="n">
-        <v>2018</v>
+        <v>2021</v>
       </c>
       <c r="G172" t="s">
-        <v>26</v>
+        <v>44</v>
       </c>
       <c r="H172" t="s">
-        <v>76</v>
+        <v>68</v>
       </c>
     </row>
     <row r="173">
@@ -5063,25 +5081,25 @@
         <v>73</v>
       </c>
       <c r="B173" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="C173" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D173" t="n">
-        <v>0.791245271940118</v>
+        <v>1072852</v>
       </c>
       <c r="E173" t="s">
-        <v>81</v>
+        <v>75</v>
       </c>
       <c r="F173" t="n">
-        <v>2018</v>
+        <v>2015</v>
       </c>
       <c r="G173" t="s">
-        <v>26</v>
+        <v>44</v>
       </c>
       <c r="H173" t="s">
-        <v>76</v>
+        <v>68</v>
       </c>
     </row>
     <row r="174">
@@ -5089,25 +5107,25 @@
         <v>73</v>
       </c>
       <c r="B174" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="C174" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D174" t="n">
-        <v>0.81384139803138</v>
+        <v>650399.1079245</v>
       </c>
       <c r="E174" t="s">
-        <v>81</v>
+        <v>75</v>
       </c>
       <c r="F174" t="n">
-        <v>2018</v>
+        <v>2021</v>
       </c>
       <c r="G174" t="s">
-        <v>26</v>
+        <v>44</v>
       </c>
       <c r="H174" t="s">
-        <v>76</v>
+        <v>68</v>
       </c>
     </row>
     <row r="175">
@@ -5115,25 +5133,753 @@
         <v>73</v>
       </c>
       <c r="B175" t="s">
+        <v>78</v>
+      </c>
+      <c r="C175" t="s">
+        <v>10</v>
+      </c>
+      <c r="D175" t="n">
+        <v>1970906.38765</v>
+      </c>
+      <c r="E175" t="s">
+        <v>75</v>
+      </c>
+      <c r="F175" t="n">
+        <v>2021</v>
+      </c>
+      <c r="G175" t="s">
+        <v>44</v>
+      </c>
+      <c r="H175" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="s">
+        <v>79</v>
+      </c>
+      <c r="B176" t="s">
         <v>80</v>
       </c>
-      <c r="C175" t="s">
+      <c r="C176" t="s">
+        <v>10</v>
+      </c>
+      <c r="D176" t="n">
+        <v>1.00972599678899</v>
+      </c>
+      <c r="E176" t="s">
+        <v>81</v>
+      </c>
+      <c r="F176" t="n">
+        <v>2018</v>
+      </c>
+      <c r="G176" t="s">
+        <v>26</v>
+      </c>
+      <c r="H176" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="s">
+        <v>79</v>
+      </c>
+      <c r="B177" t="s">
+        <v>80</v>
+      </c>
+      <c r="C177" t="s">
+        <v>14</v>
+      </c>
+      <c r="D177" t="n">
+        <v>1.38463301489268</v>
+      </c>
+      <c r="E177" t="s">
+        <v>81</v>
+      </c>
+      <c r="F177" t="n">
+        <v>2018</v>
+      </c>
+      <c r="G177" t="s">
+        <v>26</v>
+      </c>
+      <c r="H177" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="s">
+        <v>79</v>
+      </c>
+      <c r="B178" t="s">
+        <v>80</v>
+      </c>
+      <c r="C178" t="s">
+        <v>15</v>
+      </c>
+      <c r="D178" t="n">
+        <v>1.01159962166824</v>
+      </c>
+      <c r="E178" t="s">
+        <v>81</v>
+      </c>
+      <c r="F178" t="n">
+        <v>2018</v>
+      </c>
+      <c r="G178" t="s">
+        <v>26</v>
+      </c>
+      <c r="H178" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="s">
+        <v>79</v>
+      </c>
+      <c r="B179" t="s">
+        <v>80</v>
+      </c>
+      <c r="C179" t="s">
+        <v>16</v>
+      </c>
+      <c r="D179" t="n">
+        <v>1.34113695951916</v>
+      </c>
+      <c r="E179" t="s">
+        <v>81</v>
+      </c>
+      <c r="F179" t="n">
+        <v>2018</v>
+      </c>
+      <c r="G179" t="s">
+        <v>26</v>
+      </c>
+      <c r="H179" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="s">
+        <v>79</v>
+      </c>
+      <c r="B180" t="s">
+        <v>80</v>
+      </c>
+      <c r="C180" t="s">
+        <v>17</v>
+      </c>
+      <c r="D180" t="n">
+        <v>1.51107677264798</v>
+      </c>
+      <c r="E180" t="s">
+        <v>81</v>
+      </c>
+      <c r="F180" t="n">
+        <v>2018</v>
+      </c>
+      <c r="G180" t="s">
+        <v>26</v>
+      </c>
+      <c r="H180" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="s">
+        <v>79</v>
+      </c>
+      <c r="B181" t="s">
+        <v>80</v>
+      </c>
+      <c r="C181" t="s">
+        <v>18</v>
+      </c>
+      <c r="D181" t="n">
+        <v>1.10028979595841</v>
+      </c>
+      <c r="E181" t="s">
+        <v>81</v>
+      </c>
+      <c r="F181" t="n">
+        <v>2018</v>
+      </c>
+      <c r="G181" t="s">
+        <v>26</v>
+      </c>
+      <c r="H181" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="s">
+        <v>79</v>
+      </c>
+      <c r="B182" t="s">
+        <v>80</v>
+      </c>
+      <c r="C182" t="s">
         <v>19</v>
       </c>
-      <c r="D175" t="n">
+      <c r="D182" t="n">
+        <v>2.67558022226578</v>
+      </c>
+      <c r="E182" t="s">
+        <v>81</v>
+      </c>
+      <c r="F182" t="n">
+        <v>2018</v>
+      </c>
+      <c r="G182" t="s">
+        <v>26</v>
+      </c>
+      <c r="H182" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="s">
+        <v>79</v>
+      </c>
+      <c r="B183" t="s">
+        <v>83</v>
+      </c>
+      <c r="C183" t="s">
+        <v>10</v>
+      </c>
+      <c r="D183" t="n">
+        <v>1.35461522604007</v>
+      </c>
+      <c r="E183" t="s">
+        <v>81</v>
+      </c>
+      <c r="F183" t="n">
+        <v>2018</v>
+      </c>
+      <c r="G183" t="s">
+        <v>26</v>
+      </c>
+      <c r="H183" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="s">
+        <v>79</v>
+      </c>
+      <c r="B184" t="s">
+        <v>83</v>
+      </c>
+      <c r="C184" t="s">
+        <v>14</v>
+      </c>
+      <c r="D184" t="n">
+        <v>1.33052676362134</v>
+      </c>
+      <c r="E184" t="s">
+        <v>81</v>
+      </c>
+      <c r="F184" t="n">
+        <v>2018</v>
+      </c>
+      <c r="G184" t="s">
+        <v>26</v>
+      </c>
+      <c r="H184" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="s">
+        <v>79</v>
+      </c>
+      <c r="B185" t="s">
+        <v>83</v>
+      </c>
+      <c r="C185" t="s">
+        <v>15</v>
+      </c>
+      <c r="D185" t="n">
+        <v>1.44639724826724</v>
+      </c>
+      <c r="E185" t="s">
+        <v>81</v>
+      </c>
+      <c r="F185" t="n">
+        <v>2018</v>
+      </c>
+      <c r="G185" t="s">
+        <v>26</v>
+      </c>
+      <c r="H185" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="s">
+        <v>79</v>
+      </c>
+      <c r="B186" t="s">
+        <v>83</v>
+      </c>
+      <c r="C186" t="s">
+        <v>16</v>
+      </c>
+      <c r="D186" t="n">
+        <v>1.50003805694812</v>
+      </c>
+      <c r="E186" t="s">
+        <v>81</v>
+      </c>
+      <c r="F186" t="n">
+        <v>2018</v>
+      </c>
+      <c r="G186" t="s">
+        <v>26</v>
+      </c>
+      <c r="H186" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="s">
+        <v>79</v>
+      </c>
+      <c r="B187" t="s">
+        <v>83</v>
+      </c>
+      <c r="C187" t="s">
+        <v>17</v>
+      </c>
+      <c r="D187" t="n">
+        <v>1.67606087093891</v>
+      </c>
+      <c r="E187" t="s">
+        <v>81</v>
+      </c>
+      <c r="F187" t="n">
+        <v>2018</v>
+      </c>
+      <c r="G187" t="s">
+        <v>26</v>
+      </c>
+      <c r="H187" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="s">
+        <v>79</v>
+      </c>
+      <c r="B188" t="s">
+        <v>83</v>
+      </c>
+      <c r="C188" t="s">
+        <v>18</v>
+      </c>
+      <c r="D188" t="n">
+        <v>1.40536722167565</v>
+      </c>
+      <c r="E188" t="s">
+        <v>81</v>
+      </c>
+      <c r="F188" t="n">
+        <v>2018</v>
+      </c>
+      <c r="G188" t="s">
+        <v>26</v>
+      </c>
+      <c r="H188" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="s">
+        <v>79</v>
+      </c>
+      <c r="B189" t="s">
+        <v>83</v>
+      </c>
+      <c r="C189" t="s">
+        <v>19</v>
+      </c>
+      <c r="D189" t="n">
+        <v>1.32103699624993</v>
+      </c>
+      <c r="E189" t="s">
+        <v>81</v>
+      </c>
+      <c r="F189" t="n">
+        <v>2018</v>
+      </c>
+      <c r="G189" t="s">
+        <v>26</v>
+      </c>
+      <c r="H189" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="s">
+        <v>79</v>
+      </c>
+      <c r="B190" t="s">
+        <v>84</v>
+      </c>
+      <c r="C190" t="s">
+        <v>10</v>
+      </c>
+      <c r="D190" t="n">
+        <v>41.2818689801426</v>
+      </c>
+      <c r="E190" t="s">
+        <v>85</v>
+      </c>
+      <c r="F190" t="n">
+        <v>2018</v>
+      </c>
+      <c r="G190" t="s">
+        <v>26</v>
+      </c>
+      <c r="H190" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="s">
+        <v>79</v>
+      </c>
+      <c r="B191" t="s">
+        <v>84</v>
+      </c>
+      <c r="C191" t="s">
+        <v>14</v>
+      </c>
+      <c r="D191" t="n">
+        <v>6.58456873124472</v>
+      </c>
+      <c r="E191" t="s">
+        <v>85</v>
+      </c>
+      <c r="F191" t="n">
+        <v>2018</v>
+      </c>
+      <c r="G191" t="s">
+        <v>26</v>
+      </c>
+      <c r="H191" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="s">
+        <v>79</v>
+      </c>
+      <c r="B192" t="s">
+        <v>84</v>
+      </c>
+      <c r="C192" t="s">
+        <v>15</v>
+      </c>
+      <c r="D192" t="n">
+        <v>17.2338509998643</v>
+      </c>
+      <c r="E192" t="s">
+        <v>85</v>
+      </c>
+      <c r="F192" t="n">
+        <v>2018</v>
+      </c>
+      <c r="G192" t="s">
+        <v>26</v>
+      </c>
+      <c r="H192" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="s">
+        <v>79</v>
+      </c>
+      <c r="B193" t="s">
+        <v>84</v>
+      </c>
+      <c r="C193" t="s">
+        <v>16</v>
+      </c>
+      <c r="D193" t="n">
+        <v>27.3242498786245</v>
+      </c>
+      <c r="E193" t="s">
+        <v>85</v>
+      </c>
+      <c r="F193" t="n">
+        <v>2018</v>
+      </c>
+      <c r="G193" t="s">
+        <v>26</v>
+      </c>
+      <c r="H193" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="s">
+        <v>79</v>
+      </c>
+      <c r="B194" t="s">
+        <v>84</v>
+      </c>
+      <c r="C194" t="s">
+        <v>17</v>
+      </c>
+      <c r="D194" t="n">
+        <v>78.7763190160058</v>
+      </c>
+      <c r="E194" t="s">
+        <v>85</v>
+      </c>
+      <c r="F194" t="n">
+        <v>2018</v>
+      </c>
+      <c r="G194" t="s">
+        <v>26</v>
+      </c>
+      <c r="H194" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="s">
+        <v>79</v>
+      </c>
+      <c r="B195" t="s">
+        <v>84</v>
+      </c>
+      <c r="C195" t="s">
+        <v>18</v>
+      </c>
+      <c r="D195" t="n">
+        <v>16.4076079379625</v>
+      </c>
+      <c r="E195" t="s">
+        <v>85</v>
+      </c>
+      <c r="F195" t="n">
+        <v>2018</v>
+      </c>
+      <c r="G195" t="s">
+        <v>26</v>
+      </c>
+      <c r="H195" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="s">
+        <v>79</v>
+      </c>
+      <c r="B196" t="s">
+        <v>84</v>
+      </c>
+      <c r="C196" t="s">
+        <v>19</v>
+      </c>
+      <c r="D196" t="n">
+        <v>25.3412219653864</v>
+      </c>
+      <c r="E196" t="s">
+        <v>85</v>
+      </c>
+      <c r="F196" t="n">
+        <v>2018</v>
+      </c>
+      <c r="G196" t="s">
+        <v>26</v>
+      </c>
+      <c r="H196" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="s">
+        <v>79</v>
+      </c>
+      <c r="B197" t="s">
+        <v>86</v>
+      </c>
+      <c r="C197" t="s">
+        <v>10</v>
+      </c>
+      <c r="D197" t="n">
+        <v>0.87377430071436</v>
+      </c>
+      <c r="E197" t="s">
+        <v>87</v>
+      </c>
+      <c r="F197" t="n">
+        <v>2018</v>
+      </c>
+      <c r="G197" t="s">
+        <v>26</v>
+      </c>
+      <c r="H197" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="s">
+        <v>79</v>
+      </c>
+      <c r="B198" t="s">
+        <v>86</v>
+      </c>
+      <c r="C198" t="s">
+        <v>14</v>
+      </c>
+      <c r="D198" t="n">
+        <v>0.882565776633652</v>
+      </c>
+      <c r="E198" t="s">
+        <v>87</v>
+      </c>
+      <c r="F198" t="n">
+        <v>2018</v>
+      </c>
+      <c r="G198" t="s">
+        <v>26</v>
+      </c>
+      <c r="H198" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="s">
+        <v>79</v>
+      </c>
+      <c r="B199" t="s">
+        <v>86</v>
+      </c>
+      <c r="C199" t="s">
+        <v>15</v>
+      </c>
+      <c r="D199" t="n">
+        <v>0.874031286778138</v>
+      </c>
+      <c r="E199" t="s">
+        <v>87</v>
+      </c>
+      <c r="F199" t="n">
+        <v>2018</v>
+      </c>
+      <c r="G199" t="s">
+        <v>26</v>
+      </c>
+      <c r="H199" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="s">
+        <v>79</v>
+      </c>
+      <c r="B200" t="s">
+        <v>86</v>
+      </c>
+      <c r="C200" t="s">
+        <v>16</v>
+      </c>
+      <c r="D200" t="n">
+        <v>0.7700582389548</v>
+      </c>
+      <c r="E200" t="s">
+        <v>87</v>
+      </c>
+      <c r="F200" t="n">
+        <v>2018</v>
+      </c>
+      <c r="G200" t="s">
+        <v>26</v>
+      </c>
+      <c r="H200" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="s">
+        <v>79</v>
+      </c>
+      <c r="B201" t="s">
+        <v>86</v>
+      </c>
+      <c r="C201" t="s">
+        <v>17</v>
+      </c>
+      <c r="D201" t="n">
+        <v>0.791245271940118</v>
+      </c>
+      <c r="E201" t="s">
+        <v>87</v>
+      </c>
+      <c r="F201" t="n">
+        <v>2018</v>
+      </c>
+      <c r="G201" t="s">
+        <v>26</v>
+      </c>
+      <c r="H201" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="s">
+        <v>79</v>
+      </c>
+      <c r="B202" t="s">
+        <v>86</v>
+      </c>
+      <c r="C202" t="s">
+        <v>18</v>
+      </c>
+      <c r="D202" t="n">
+        <v>0.81384139803138</v>
+      </c>
+      <c r="E202" t="s">
+        <v>87</v>
+      </c>
+      <c r="F202" t="n">
+        <v>2018</v>
+      </c>
+      <c r="G202" t="s">
+        <v>26</v>
+      </c>
+      <c r="H202" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="s">
+        <v>79</v>
+      </c>
+      <c r="B203" t="s">
+        <v>86</v>
+      </c>
+      <c r="C203" t="s">
+        <v>19</v>
+      </c>
+      <c r="D203" t="n">
         <v>0.899495827765645</v>
       </c>
-      <c r="E175" t="s">
-        <v>81</v>
-      </c>
-      <c r="F175" t="n">
+      <c r="E203" t="s">
+        <v>87</v>
+      </c>
+      <c r="F203" t="n">
         <v>2018</v>
       </c>
-      <c r="G175" t="s">
-        <v>26</v>
-      </c>
-      <c r="H175" t="s">
-        <v>76</v>
+      <c r="G203" t="s">
+        <v>26</v>
+      </c>
+      <c r="H203" t="s">
+        <v>82</v>
       </c>
     </row>
   </sheetData>

</xml_diff>